<commit_message>
Build out explicit Free Cash Flow / share bridge
Replace the single-line FCF rows with a full, line-by-line build
(rows 114-128) addressing the model's "Need to build out FCF/Share" TODO:

  Net Income
  (+) D&A, intangible amortization, SBC, debenture amortization
  (+/-) Decrease / (increase) in net working capital
  (-) Capital expenditures
  = Free Cash Flow  -> % growth, FCF margin
  / Diluted weighted-average shares
  = Free Cash Flow per Share -> % growth, FCF yield (FX-adjusted to the
    CAD share price)

Every component links to its source line so the bridge is fully
traceable. FCF/share: $1.49 (2026) rising to $2.28 (2030); FCF yield
7.4% to 11.2% on the current C$28.86 price. Cached values rewritten for
all formula cells.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LQHeLrCxSK9A3QCVVG7xC5
</commit_message>
<xml_diff>
--- a/EFN_Modelv2.xlsx
+++ b/EFN_Modelv2.xlsx
@@ -499,7 +499,7 @@
     <xf numFmtId="9" fontId="33" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="34" fillId="9" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="418">
+  <cellXfs count="420">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1078,6 +1078,8 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1584,7 +1586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB113"/>
+  <dimension ref="A1:AB128"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col width="10.5703125" customWidth="1" style="305" min="1" max="1"/>
@@ -7352,16 +7354,8 @@
       </c>
     </row>
     <row r="94" outlineLevel="1" s="20">
-      <c r="B94" s="89" t="inlineStr">
-        <is>
-          <t>Free Cash Flow</t>
-        </is>
-      </c>
-      <c r="C94" s="307" t="inlineStr">
-        <is>
-          <t>$</t>
-        </is>
-      </c>
+      <c r="B94" s="89" t="n"/>
+      <c r="C94" s="307" t="n"/>
       <c r="D94" s="351" t="n"/>
       <c r="E94" s="351" t="n"/>
       <c r="F94" s="351" t="n"/>
@@ -7373,42 +7367,19 @@
       <c r="L94" s="351" t="n"/>
       <c r="M94" s="351" t="n"/>
       <c r="N94" s="351" t="n"/>
-      <c r="O94" s="197">
-        <f>O55+O26+O39+O32+O29-O87-O89</f>
-        <v>593.4763151699973</v>
-      </c>
+      <c r="O94" s="197" t="n"/>
       <c r="P94" s="351" t="n"/>
       <c r="Q94" s="351" t="n"/>
       <c r="R94" s="351" t="n"/>
       <c r="S94" s="351" t="n"/>
-      <c r="T94" s="197">
-        <f>T55+T26+T39+T32+T29-T87-T89</f>
-        <v>695.0768177351315</v>
-      </c>
-      <c r="U94" s="197">
-        <f>U55+U26+U39+U32+U29-U87-U89</f>
-        <v>769.557509745625</v>
-      </c>
-      <c r="V94" s="197">
-        <f>V55+V26+V39+V32+V29-V87-V89</f>
-        <v>840.0090199037589</v>
-      </c>
-      <c r="W94" s="197">
-        <f>W55+W26+W39+W32+W29-W87-W89</f>
-        <v>907.8432817646716</v>
-      </c>
+      <c r="T94" s="197" t="n"/>
+      <c r="U94" s="197" t="n"/>
+      <c r="V94" s="197" t="n"/>
+      <c r="W94" s="197" t="n"/>
     </row>
     <row r="95" outlineLevel="1" s="20">
-      <c r="B95" s="89" t="inlineStr">
-        <is>
-          <t>FCF per Share</t>
-        </is>
-      </c>
-      <c r="C95" s="307" t="inlineStr">
-        <is>
-          <t>$</t>
-        </is>
-      </c>
+      <c r="B95" s="89" t="n"/>
+      <c r="C95" s="307" t="n"/>
       <c r="D95" s="351" t="n"/>
       <c r="E95" s="351" t="n"/>
       <c r="F95" s="351" t="n"/>
@@ -7420,42 +7391,19 @@
       <c r="L95" s="351" t="n"/>
       <c r="M95" s="351" t="n"/>
       <c r="N95" s="351" t="n"/>
-      <c r="O95" s="197">
-        <f>O94/O100</f>
-        <v>1.4926632258405288</v>
-      </c>
+      <c r="O95" s="197" t="n"/>
       <c r="P95" s="351" t="n"/>
       <c r="Q95" s="351" t="n"/>
       <c r="R95" s="351" t="n"/>
       <c r="S95" s="351" t="n"/>
-      <c r="T95" s="197">
-        <f>T94/T100</f>
-        <v>1.7486223354020698</v>
-      </c>
-      <c r="U95" s="197">
-        <f>U94/U100</f>
-        <v>1.935610026081336</v>
-      </c>
-      <c r="V95" s="197">
-        <f>V94/V100</f>
-        <v>2.1128114017910353</v>
-      </c>
-      <c r="W95" s="197">
-        <f>W94/W100</f>
-        <v>2.283429810041265</v>
-      </c>
+      <c r="T95" s="197" t="n"/>
+      <c r="U95" s="197" t="n"/>
+      <c r="V95" s="197" t="n"/>
+      <c r="W95" s="197" t="n"/>
     </row>
     <row r="96" outlineLevel="1" s="20">
-      <c r="B96" s="89" t="inlineStr">
-        <is>
-          <t>FCF Margin</t>
-        </is>
-      </c>
-      <c r="C96" s="307" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+      <c r="B96" s="89" t="n"/>
+      <c r="C96" s="307" t="n"/>
       <c r="D96" s="351" t="n"/>
       <c r="E96" s="351" t="n"/>
       <c r="F96" s="351" t="n"/>
@@ -7467,30 +7415,15 @@
       <c r="L96" s="351" t="n"/>
       <c r="M96" s="351" t="n"/>
       <c r="N96" s="351" t="n"/>
-      <c r="O96" s="353">
-        <f>O94/O17</f>
-        <v>0.45210708763780955</v>
-      </c>
+      <c r="O96" s="353" t="n"/>
       <c r="P96" s="351" t="n"/>
       <c r="Q96" s="351" t="n"/>
       <c r="R96" s="351" t="n"/>
       <c r="S96" s="351" t="n"/>
-      <c r="T96" s="353">
-        <f>T94/T17</f>
-        <v>0.49292893634558277</v>
-      </c>
-      <c r="U96" s="353">
-        <f>U94/U17</f>
-        <v>0.5024671042595343</v>
-      </c>
-      <c r="V96" s="353">
-        <f>V94/V17</f>
-        <v>0.5049238035431176</v>
-      </c>
-      <c r="W96" s="353">
-        <f>W94/W17</f>
-        <v>0.5080155921363421</v>
-      </c>
+      <c r="T96" s="353" t="n"/>
+      <c r="U96" s="353" t="n"/>
+      <c r="V96" s="353" t="n"/>
+      <c r="W96" s="353" t="n"/>
     </row>
     <row r="97" ht="14.45" customHeight="1" s="20">
       <c r="B97" s="320" t="n"/>
@@ -8041,17 +7974,410 @@
       <c r="AB111" s="330" t="n"/>
     </row>
     <row r="112">
-      <c r="B112" s="325" t="inlineStr">
-        <is>
-          <t>Need to build out FCF/Share</t>
-        </is>
-      </c>
+      <c r="B112" s="325" t="n"/>
     </row>
     <row r="113">
       <c r="B113" s="307" t="inlineStr">
         <is>
           <t>Share buybacks</t>
         </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="82" t="inlineStr">
+        <is>
+          <t>Free Cash Flow Build</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="307" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="O115" s="418">
+        <f>O55</f>
+        <v>493.6006060978542</v>
+      </c>
+      <c r="T115" s="418">
+        <f>T55</f>
+        <v>539.0756351169435</v>
+      </c>
+      <c r="U115" s="418">
+        <f>U55</f>
+        <v>594.5654048790257</v>
+      </c>
+      <c r="V115" s="418">
+        <f>V55</f>
+        <v>656.8006281804242</v>
+      </c>
+      <c r="W115" s="418">
+        <f>W55</f>
+        <v>714.9485348876021</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="307" t="inlineStr">
+        <is>
+          <t>(+) Depreciation &amp; amortization</t>
+        </is>
+      </c>
+      <c r="O116" s="418">
+        <f>O26</f>
+        <v>71.43155324828221</v>
+      </c>
+      <c r="T116" s="418">
+        <f>T26</f>
+        <v>77.16377781143325</v>
+      </c>
+      <c r="U116" s="418">
+        <f>U26</f>
+        <v>83.81050106647312</v>
+      </c>
+      <c r="V116" s="418">
+        <f>V26</f>
+        <v>91.03808116009077</v>
+      </c>
+      <c r="W116" s="418">
+        <f>W26</f>
+        <v>97.79098780536819</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" s="307" t="inlineStr">
+        <is>
+          <t>(+) Amortization of intangibles</t>
+        </is>
+      </c>
+      <c r="O117" s="418">
+        <f>O39</f>
+        <v>36.432945434556316</v>
+      </c>
+      <c r="T117" s="418">
+        <f>T39</f>
+        <v>38.938839105828066</v>
+      </c>
+      <c r="U117" s="418">
+        <f>U39</f>
+        <v>42.29294766232509</v>
+      </c>
+      <c r="V117" s="418">
+        <f>V39</f>
+        <v>45.94017161081564</v>
+      </c>
+      <c r="W117" s="418">
+        <f>W39</f>
+        <v>49.347863053809945</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="307" t="inlineStr">
+        <is>
+          <t>(+) Share-based compensation</t>
+        </is>
+      </c>
+      <c r="O118" s="418">
+        <f>O32</f>
+        <v>43.997826787093494</v>
+      </c>
+      <c r="T118" s="418">
+        <f>T32</f>
+        <v>49.16343402930033</v>
+      </c>
+      <c r="U118" s="418">
+        <f>U32</f>
+        <v>53.39826738671731</v>
+      </c>
+      <c r="V118" s="418">
+        <f>V32</f>
+        <v>58.00318263584351</v>
+      </c>
+      <c r="W118" s="418">
+        <f>W32</f>
+        <v>62.30566872163918</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" s="307" t="inlineStr">
+        <is>
+          <t>(+) Amortization of debenture discount</t>
+        </is>
+      </c>
+      <c r="O119" s="418">
+        <f>O29</f>
+        <v>0.0</v>
+      </c>
+      <c r="T119" s="418">
+        <f>T29</f>
+        <v>0.0</v>
+      </c>
+      <c r="U119" s="418">
+        <f>U29</f>
+        <v>0.0</v>
+      </c>
+      <c r="V119" s="418">
+        <f>V29</f>
+        <v>0.0</v>
+      </c>
+      <c r="W119" s="418">
+        <f>W29</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="307" t="inlineStr">
+        <is>
+          <t>(+/-) Decrease / (increase) in net working capital</t>
+        </is>
+      </c>
+      <c r="O120" s="418">
+        <f>-O87</f>
+        <v>28.013383602211093</v>
+      </c>
+      <c r="T120" s="418">
+        <f>-T87</f>
+        <v>70.73513167162628</v>
+      </c>
+      <c r="U120" s="418">
+        <f>-U87</f>
+        <v>75.49038875108386</v>
+      </c>
+      <c r="V120" s="418">
+        <f>-V87</f>
+        <v>68.22695631658485</v>
+      </c>
+      <c r="W120" s="418">
+        <f>-W87</f>
+        <v>63.450227296252024</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="307" t="inlineStr">
+        <is>
+          <t>(-) Capital expenditures</t>
+        </is>
+      </c>
+      <c r="O121" s="418">
+        <f>-O89</f>
+        <v>-80.0</v>
+      </c>
+      <c r="T121" s="418">
+        <f>-T89</f>
+        <v>-80.0</v>
+      </c>
+      <c r="U121" s="418">
+        <f>-U89</f>
+        <v>-80.0</v>
+      </c>
+      <c r="V121" s="418">
+        <f>-V89</f>
+        <v>-80.0</v>
+      </c>
+      <c r="W121" s="418">
+        <f>-W89</f>
+        <v>-80.0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="307" t="inlineStr">
+        <is>
+          <t>Free Cash Flow</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="O122" s="418">
+        <f>SUM(O115:O121)</f>
+        <v>593.4763151699973</v>
+      </c>
+      <c r="T122" s="418">
+        <f>SUM(T115:T121)</f>
+        <v>695.0768177351315</v>
+      </c>
+      <c r="U122" s="418">
+        <f>SUM(U115:U121)</f>
+        <v>769.557509745625</v>
+      </c>
+      <c r="V122" s="418">
+        <f>SUM(V115:V121)</f>
+        <v>840.0090199037589</v>
+      </c>
+      <c r="W122" s="418">
+        <f>SUM(W115:W121)</f>
+        <v>907.8432817646716</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="307" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   % growth</t>
+        </is>
+      </c>
+      <c r="T123" s="344">
+        <f>T122/O122-1</f>
+        <v>0.17119554726633268</v>
+      </c>
+      <c r="U123" s="344">
+        <f>U122/T122-1</f>
+        <v>0.10715461961914463</v>
+      </c>
+      <c r="V123" s="344">
+        <f>V122/U122-1</f>
+        <v>0.09154807700001721</v>
+      </c>
+      <c r="W123" s="344">
+        <f>W122/V122-1</f>
+        <v>0.0807542065068354</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" s="307" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   FCF margin (% net revenue)</t>
+        </is>
+      </c>
+      <c r="O124" s="344">
+        <f>O122/O17</f>
+        <v>0.45210708763780955</v>
+      </c>
+      <c r="T124" s="344">
+        <f>T122/T17</f>
+        <v>0.49292893634558277</v>
+      </c>
+      <c r="U124" s="344">
+        <f>U122/U17</f>
+        <v>0.5024671042595343</v>
+      </c>
+      <c r="V124" s="344">
+        <f>V122/V17</f>
+        <v>0.5049238035431176</v>
+      </c>
+      <c r="W124" s="344">
+        <f>W122/W17</f>
+        <v>0.5080155921363421</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="307" t="inlineStr">
+        <is>
+          <t>Diluted weighted-average shares</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="O125" s="418">
+        <f>O100</f>
+        <v>397.5955894778655</v>
+      </c>
+      <c r="T125" s="418">
+        <f>T100</f>
+        <v>397.4996794120835</v>
+      </c>
+      <c r="U125" s="418">
+        <f>U100</f>
+        <v>397.5787991259803</v>
+      </c>
+      <c r="V125" s="418">
+        <f>V100</f>
+        <v>397.5787991259803</v>
+      </c>
+      <c r="W125" s="418">
+        <f>W100</f>
+        <v>397.5787991259803</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" s="307" t="inlineStr">
+        <is>
+          <t>Free Cash Flow per Share</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="O126" s="419">
+        <f>O122/O125</f>
+        <v>1.4926632258405288</v>
+      </c>
+      <c r="T126" s="419">
+        <f>T122/T125</f>
+        <v>1.7486223354020698</v>
+      </c>
+      <c r="U126" s="419">
+        <f>U122/U125</f>
+        <v>1.935610026081336</v>
+      </c>
+      <c r="V126" s="419">
+        <f>V122/V125</f>
+        <v>2.1128114017910353</v>
+      </c>
+      <c r="W126" s="419">
+        <f>W122/W125</f>
+        <v>2.283429810041265</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" s="307" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   % growth</t>
+        </is>
+      </c>
+      <c r="T127" s="344">
+        <f>T126/O126-1</f>
+        <v>0.17147813728539374</v>
+      </c>
+      <c r="U127" s="344">
+        <f>U126/T126-1</f>
+        <v>0.10693429158118994</v>
+      </c>
+      <c r="V127" s="344">
+        <f>V126/U126-1</f>
+        <v>0.09154807700001721</v>
+      </c>
+      <c r="W127" s="344">
+        <f>W126/V126-1</f>
+        <v>0.0807542065068354</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="B128" s="307" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   FCF yield (on current price)</t>
+        </is>
+      </c>
+      <c r="O128" s="344">
+        <f>O126*O110/O109</f>
+        <v>0.07350564714360913</v>
+      </c>
+      <c r="T128" s="344">
+        <f>T126*T110/T109</f>
+        <v>0.08611025859575266</v>
+      </c>
+      <c r="U128" s="344">
+        <f>U126*U110/U109</f>
+        <v>0.09531839809656253</v>
+      </c>
+      <c r="V128" s="344">
+        <f>V126*V110/V109</f>
+        <v>0.10404461414502493</v>
+      </c>
+      <c r="W128" s="344">
+        <f>W126*W110/W109</f>
+        <v>0.11244665440161629</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add quarterly FCF/share build (Q2'26-Q4'27)
Extend the Free Cash Flow bridge across the quarterly forecast columns
in addition to the annual columns. Adds quarterly capital expenditures
(rows 89: $20M/quarter = annual $80M / 4) so quarterly FCF is complete.

The bridge lines (net income through FCF, FCF margin, diluted shares,
FCF per share) now populate Q2'26E-Q4'27E alongside the annual columns;
growth and FCF-yield lines remain annual-only as those are annual
concepts.

Note: Q2'26 FCF is elevated (~$297M) because the Q1'26 payables dip
(actual) reverses in Q2, landing a one-time ~$161M working-capital
source that quarter. The annual view nets this against the Q1'26
paydown, so 2026 annual FCF is unaffected ($593M).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LQHeLrCxSK9A3QCVVG7xC5
</commit_message>
<xml_diff>
--- a/EFN_Modelv2.xlsx
+++ b/EFN_Modelv2.xlsx
@@ -7085,16 +7085,30 @@
       <c r="I89" s="303" t="n"/>
       <c r="J89" s="303" t="n"/>
       <c r="K89" s="304" t="n"/>
-      <c r="L89" s="303" t="n"/>
-      <c r="M89" s="303" t="n"/>
-      <c r="N89" s="303" t="n"/>
+      <c r="L89" s="303" t="n">
+        <v>20</v>
+      </c>
+      <c r="M89" s="303" t="n">
+        <v>20</v>
+      </c>
+      <c r="N89" s="303" t="n">
+        <v>20</v>
+      </c>
       <c r="O89" s="238" t="n">
         <v>80</v>
       </c>
-      <c r="P89" s="238" t="n"/>
-      <c r="Q89" s="238" t="n"/>
-      <c r="R89" s="238" t="n"/>
-      <c r="S89" s="238" t="n"/>
+      <c r="P89" s="238" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q89" s="238" t="n">
+        <v>20</v>
+      </c>
+      <c r="R89" s="238" t="n">
+        <v>20</v>
+      </c>
+      <c r="S89" s="238" t="n">
+        <v>20</v>
+      </c>
       <c r="T89" s="238" t="n">
         <v>80</v>
       </c>
@@ -8001,10 +8015,38 @@
           <t>$</t>
         </is>
       </c>
+      <c r="L115" s="418">
+        <f>L55</f>
+        <v>118.56365419179409</v>
+      </c>
+      <c r="M115" s="418">
+        <f>M55</f>
+        <v>127.39838589081758</v>
+      </c>
+      <c r="N115" s="418">
+        <f>N55</f>
+        <v>129.0965660152424</v>
+      </c>
       <c r="O115" s="418">
         <f>O55</f>
         <v>493.6006060978542</v>
       </c>
+      <c r="P115" s="418">
+        <f>P55</f>
+        <v>122.14335969256284</v>
+      </c>
+      <c r="Q115" s="418">
+        <f>Q55</f>
+        <v>130.3038561893571</v>
+      </c>
+      <c r="R115" s="418">
+        <f>R55</f>
+        <v>139.4374090825442</v>
+      </c>
+      <c r="S115" s="418">
+        <f>S55</f>
+        <v>140.0734046350983</v>
+      </c>
       <c r="T115" s="418">
         <f>T55</f>
         <v>539.0756351169435</v>
@@ -8028,10 +8070,38 @@
           <t>(+) Depreciation &amp; amortization</t>
         </is>
       </c>
+      <c r="L116" s="418">
+        <f>L26</f>
+        <v>17.19838588667246</v>
+      </c>
+      <c r="M116" s="418">
+        <f>M26</f>
+        <v>18.47991795483252</v>
+      </c>
+      <c r="N116" s="418">
+        <f>N26</f>
+        <v>18.726249406777224</v>
+      </c>
       <c r="O116" s="418">
         <f>O26</f>
         <v>71.43155324828221</v>
       </c>
+      <c r="P116" s="418">
+        <f>P26</f>
+        <v>17.717644144884325</v>
+      </c>
+      <c r="Q116" s="418">
+        <f>Q26</f>
+        <v>18.901374257922797</v>
+      </c>
+      <c r="R116" s="418">
+        <f>R26</f>
+        <v>20.22625217471897</v>
+      </c>
+      <c r="S116" s="418">
+        <f>S26</f>
+        <v>20.318507233907162</v>
+      </c>
       <c r="T116" s="418">
         <f>T26</f>
         <v>77.16377781143325</v>
@@ -8055,10 +8125,38 @@
           <t>(+) Amortization of intangibles</t>
         </is>
       </c>
+      <c r="L117" s="418">
+        <f>L39</f>
+        <v>8.678750573327381</v>
+      </c>
+      <c r="M117" s="418">
+        <f>M39</f>
+        <v>9.32544481804138</v>
+      </c>
+      <c r="N117" s="418">
+        <f>N39</f>
+        <v>9.449750043187558</v>
+      </c>
       <c r="O117" s="418">
         <f>O39</f>
         <v>36.432945434556316</v>
       </c>
+      <c r="P117" s="418">
+        <f>P39</f>
+        <v>8.940781727637825</v>
+      </c>
+      <c r="Q117" s="418">
+        <f>Q39</f>
+        <v>9.538122574906438</v>
+      </c>
+      <c r="R117" s="418">
+        <f>R39</f>
+        <v>10.206690256533696</v>
+      </c>
+      <c r="S117" s="418">
+        <f>S39</f>
+        <v>10.253244546750103</v>
+      </c>
       <c r="T117" s="418">
         <f>T39</f>
         <v>38.938839105828066</v>
@@ -8082,10 +8180,38 @@
           <t>(+) Share-based compensation</t>
         </is>
       </c>
+      <c r="L118" s="418">
+        <f>L32</f>
+        <v>10.95762459966793</v>
+      </c>
+      <c r="M118" s="418">
+        <f>M32</f>
+        <v>11.774128392981229</v>
+      </c>
+      <c r="N118" s="418">
+        <f>N32</f>
+        <v>11.931073794444336</v>
+      </c>
       <c r="O118" s="418">
         <f>O32</f>
         <v>43.997826787093494</v>
       </c>
+      <c r="P118" s="418">
+        <f>P32</f>
+        <v>11.288460126981704</v>
+      </c>
+      <c r="Q118" s="418">
+        <f>Q32</f>
+        <v>12.042651263956342</v>
+      </c>
+      <c r="R118" s="418">
+        <f>R32</f>
+        <v>12.88677204065624</v>
+      </c>
+      <c r="S118" s="418">
+        <f>S32</f>
+        <v>12.945550597706047</v>
+      </c>
       <c r="T118" s="418">
         <f>T32</f>
         <v>49.16343402930033</v>
@@ -8109,10 +8235,38 @@
           <t>(+) Amortization of debenture discount</t>
         </is>
       </c>
+      <c r="L119" s="418">
+        <f>L29</f>
+        <v>0.0</v>
+      </c>
+      <c r="M119" s="418">
+        <f>M29</f>
+        <v>0.0</v>
+      </c>
+      <c r="N119" s="418">
+        <f>N29</f>
+        <v>0.0</v>
+      </c>
       <c r="O119" s="418">
         <f>O29</f>
         <v>0.0</v>
       </c>
+      <c r="P119" s="418">
+        <f>P29</f>
+        <v>0.0</v>
+      </c>
+      <c r="Q119" s="418">
+        <f>Q29</f>
+        <v>0.0</v>
+      </c>
+      <c r="R119" s="418">
+        <f>R29</f>
+        <v>0.0</v>
+      </c>
+      <c r="S119" s="418">
+        <f>S29</f>
+        <v>0.0</v>
+      </c>
       <c r="T119" s="418">
         <f>T29</f>
         <v>0.0</v>
@@ -8136,10 +8290,38 @@
           <t>(+/-) Decrease / (increase) in net working capital</t>
         </is>
       </c>
+      <c r="L120" s="418">
+        <f>-L87</f>
+        <v>161.453697247994</v>
+      </c>
+      <c r="M120" s="418">
+        <f>-M87</f>
+        <v>31.82667082236162</v>
+      </c>
+      <c r="N120" s="418">
+        <f>-N87</f>
+        <v>-13.487984468144532</v>
+      </c>
       <c r="O120" s="418">
         <f>-O87</f>
         <v>28.013383602211093</v>
       </c>
+      <c r="P120" s="418">
+        <f>-P87</f>
+        <v>0.9740359236727727</v>
+      </c>
+      <c r="Q120" s="418">
+        <f>-Q87</f>
+        <v>55.50048326469391</v>
+      </c>
+      <c r="R120" s="418">
+        <f>-R87</f>
+        <v>30.153452853152203</v>
+      </c>
+      <c r="S120" s="418">
+        <f>-S87</f>
+        <v>-15.892840369892838</v>
+      </c>
       <c r="T120" s="418">
         <f>-T87</f>
         <v>70.73513167162628</v>
@@ -8163,10 +8345,38 @@
           <t>(-) Capital expenditures</t>
         </is>
       </c>
+      <c r="L121" s="418">
+        <f>-L89</f>
+        <v>-20.0</v>
+      </c>
+      <c r="M121" s="418">
+        <f>-M89</f>
+        <v>-20.0</v>
+      </c>
+      <c r="N121" s="418">
+        <f>-N89</f>
+        <v>-20.0</v>
+      </c>
       <c r="O121" s="418">
         <f>-O89</f>
         <v>-80.0</v>
       </c>
+      <c r="P121" s="418">
+        <f>-P89</f>
+        <v>-20.0</v>
+      </c>
+      <c r="Q121" s="418">
+        <f>-Q89</f>
+        <v>-20.0</v>
+      </c>
+      <c r="R121" s="418">
+        <f>-R89</f>
+        <v>-20.0</v>
+      </c>
+      <c r="S121" s="418">
+        <f>-S89</f>
+        <v>-20.0</v>
+      </c>
       <c r="T121" s="418">
         <f>-T89</f>
         <v>-80.0</v>
@@ -8195,10 +8405,38 @@
           <t>$</t>
         </is>
       </c>
+      <c r="L122" s="418">
+        <f>SUM(L115:L121)</f>
+        <v>296.85211249945587</v>
+      </c>
+      <c r="M122" s="418">
+        <f>SUM(M115:M121)</f>
+        <v>178.80454787903432</v>
+      </c>
+      <c r="N122" s="418">
+        <f>SUM(N115:N121)</f>
+        <v>135.71565479150695</v>
+      </c>
       <c r="O122" s="418">
         <f>SUM(O115:O121)</f>
         <v>593.4763151699973</v>
       </c>
+      <c r="P122" s="418">
+        <f>SUM(P115:P121)</f>
+        <v>141.06428161573945</v>
+      </c>
+      <c r="Q122" s="418">
+        <f>SUM(Q115:Q121)</f>
+        <v>206.2864875508366</v>
+      </c>
+      <c r="R122" s="418">
+        <f>SUM(R115:R121)</f>
+        <v>192.91057640760533</v>
+      </c>
+      <c r="S122" s="418">
+        <f>SUM(S115:S121)</f>
+        <v>147.69786664356877</v>
+      </c>
       <c r="T122" s="418">
         <f>SUM(T115:T121)</f>
         <v>695.0768177351315</v>
@@ -8245,10 +8483,38 @@
           <t xml:space="preserve">   FCF margin (% net revenue)</t>
         </is>
       </c>
+      <c r="L124" s="344">
+        <f>L122/L17</f>
+        <v>0.9493254945583147</v>
+      </c>
+      <c r="M124" s="344">
+        <f>M122/M17</f>
+        <v>0.5321587551082835</v>
+      </c>
+      <c r="N124" s="344">
+        <f>N122/N17</f>
+        <v>0.39860416527569326</v>
+      </c>
       <c r="O124" s="344">
         <f>O122/O17</f>
         <v>0.45210708763780955</v>
       </c>
+      <c r="P124" s="344">
+        <f>P122/P17</f>
+        <v>0.4378988213907557</v>
+      </c>
+      <c r="Q124" s="344">
+        <f>Q122/Q17</f>
+        <v>0.6002609471922533</v>
+      </c>
+      <c r="R124" s="344">
+        <f>R122/R17</f>
+        <v>0.5245698318584182</v>
+      </c>
+      <c r="S124" s="344">
+        <f>S122/S17</f>
+        <v>0.3998021395902611</v>
+      </c>
       <c r="T124" s="344">
         <f>T122/T17</f>
         <v>0.49292893634558277</v>
@@ -8277,10 +8543,38 @@
           <t>mm</t>
         </is>
       </c>
+      <c r="L125" s="418">
+        <f>L100</f>
+        <v>397.2806971578966</v>
+      </c>
+      <c r="M125" s="418">
+        <f>M100</f>
+        <v>397.360202332559</v>
+      </c>
+      <c r="N125" s="418">
+        <f>N100</f>
+        <v>397.3999383527922</v>
+      </c>
       <c r="O125" s="418">
         <f>O100</f>
         <v>397.5955894778655</v>
       </c>
+      <c r="P125" s="418">
+        <f>P100</f>
+        <v>397.4396783466275</v>
+      </c>
+      <c r="Q125" s="418">
+        <f>Q100</f>
+        <v>397.4794223144621</v>
+      </c>
+      <c r="R125" s="418">
+        <f>R100</f>
+        <v>397.5191702566935</v>
+      </c>
+      <c r="S125" s="418">
+        <f>S100</f>
+        <v>397.5589221737192</v>
+      </c>
       <c r="T125" s="418">
         <f>T100</f>
         <v>397.4996794120835</v>
@@ -8309,9 +8603,37 @@
           <t>$</t>
         </is>
       </c>
+      <c r="L126" s="419">
+        <f>L122/L125</f>
+        <v>0.7472100069877645</v>
+      </c>
+      <c r="M126" s="419">
+        <f>M122/M125</f>
+        <v>0.4499810167938989</v>
+      </c>
+      <c r="N126" s="419">
+        <f>N122/N125</f>
+        <v>0.34150899809910196</v>
+      </c>
       <c r="O126" s="419">
         <f>O122/O125</f>
         <v>1.4926632258405288</v>
+      </c>
+      <c r="P126" s="419">
+        <f>P122/P125</f>
+        <v>0.3549325578225485</v>
+      </c>
+      <c r="Q126" s="419">
+        <f>Q122/Q125</f>
+        <v>0.5189865838831651</v>
+      </c>
+      <c r="R126" s="419">
+        <f>R122/R125</f>
+        <v>0.48528622225447776</v>
+      </c>
+      <c r="S126" s="419">
+        <f>S122/S125</f>
+        <v>0.3715118902023535</v>
       </c>
       <c r="T126" s="419">
         <f>T122/T125</f>

</xml_diff>